<commit_message>
Rename fields of BiLevel_Settings
</commit_message>
<xml_diff>
--- a/tests/utils/study_analyses/study_inputs/bilevel_d.xlsx
+++ b/tests/utils/study_analyses/study_inputs/bilevel_d.xlsx
@@ -5,11 +5,11 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\francois.gallard\Documents\workspace\GEMS\gems\utils\tests\study_inputs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matthias.delozzo\GEMSEO\gemseo\tests\utils\study_analyses\study_inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22755" windowHeight="6270" activeTab="4"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22755" windowHeight="6270" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet name="SA" sheetId="2" r:id="rId1"/>
@@ -68,9 +68,6 @@
     <t>Options values</t>
   </si>
   <si>
-    <t>apply_cstr_tosub_scenarios</t>
-  </si>
-  <si>
     <t>False</t>
   </si>
   <si>
@@ -117,6 +114,9 @@
   </si>
   <si>
     <t>prof</t>
+  </si>
+  <si>
+    <t>apply_constraints_to_sub_scenarios</t>
   </si>
 </sst>
 </file>
@@ -453,23 +453,23 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -497,23 +497,23 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -543,7 +543,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C2" t="s">
         <v>8</v>
@@ -551,12 +551,12 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -586,10 +586,10 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -621,24 +621,24 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C2" t="s">
         <v>8</v>
       </c>
       <c r="E2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G2" t="s">
         <v>6</v>
       </c>
       <c r="I2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="I3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -670,7 +670,7 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C2" t="s">
         <v>8</v>
@@ -679,12 +679,12 @@
         <v>6</v>
       </c>
       <c r="I2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="I3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -730,49 +730,49 @@
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C2" t="s">
         <v>8</v>
       </c>
       <c r="E2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G2" t="s">
         <v>9</v>
       </c>
       <c r="I2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="K2" t="s">
+        <v>28</v>
+      </c>
+      <c r="L2" t="s">
         <v>12</v>
-      </c>
-      <c r="L2" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="E3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="L3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="I4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="I5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>